<commit_message>
ajustado para inserir links externos
</commit_message>
<xml_diff>
--- a/docs/Cronograma_TV_Corporativa_atualizado.xlsx
+++ b/docs/Cronograma_TV_Corporativa_atualizado.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="157">
   <si>
     <t xml:space="preserve">CHECKLIST DE MELHORIAS – TV CORPORATIVA | GRUPO FLEXÍVEL</t>
   </si>
   <si>
-    <t xml:space="preserve">Atualizado em 19/06/2026  •  Registro das melhorias entregues nesta evolução do sistema</t>
+    <t xml:space="preserve">Atualizado em 22/06/2026  •  Andamento das entregas do sistema</t>
   </si>
   <si>
     <t xml:space="preserve">Nº</t>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">Backend</t>
   </si>
   <si>
-    <t xml:space="preserve">Reescrita e correção do servidor (server.py estava truncado e não executava)</t>
+    <t xml:space="preserve">Servidor central reescrito e corrigido (estava truncado, não rodava)</t>
   </si>
   <si>
     <t xml:space="preserve">Concluído</t>
@@ -62,31 +62,16 @@
     <t xml:space="preserve">19/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Servidor central voltou a funcionar</t>
-  </si>
-  <si>
     <t xml:space="preserve">Modelo de dados unificado (config / tvs / grades / barras)</t>
   </si>
   <si>
-    <t xml:space="preserve">Admin e TVs passam a usar o mesmo formato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin e TVs religados ao servidor central (fim do armazenamento isolado por navegador)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conteúdo sincroniza entre todas as telas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gravação atômica do conteúdo (evita corromper o arquivo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Servidor de produção (waitress) em vez do servidor de testes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">URLs amigáveis das TVs (/tela/&lt;nome&gt;)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ex.: /tela/recepcao</t>
+    <t xml:space="preserve">Admin e TVs sincronizando pelo servidor central</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gravação atômica do conteúdo + servidor de produção (waitress)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URLs amigáveis das TVs (/tela/&lt;slug&gt;)</t>
   </si>
   <si>
     <t xml:space="preserve">SEGURANÇA E ACESSO</t>
@@ -95,28 +80,22 @@
     <t xml:space="preserve">Segurança</t>
   </si>
   <si>
-    <t xml:space="preserve">Login com usuário e senha (senha criptografada + sessão)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acesso inicial: admin / flexivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proteção do painel e de todas as rotas de escrita</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TVs continuam públicas na rede interna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tela de login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tela de Usuários (criar, editar e remover logins)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Botões 'Trocar senha' e 'Sair' no painel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upload seguro (tipos permitidos + limite de 300 MB)</t>
+    <t xml:space="preserve">Login com usuário e senha (hash + sessão)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin / flexivel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tela de Usuários (criar, editar, remover) + trocar senha + sair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upload seguro (tipos permitidos + limite de tamanho)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave de API (notícias) movida para .env, fora do Git</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">ESTRUTURA E IMPLANTAÇÃO</t>
@@ -125,25 +104,16 @@
     <t xml:space="preserve">Estrutura</t>
   </si>
   <si>
-    <t xml:space="preserve">Reorganização das pastas (backend / frontend / data / uploads / docs...)</t>
+    <t xml:space="preserve">Reorganização das pastas do projeto</t>
   </si>
   <si>
     <t xml:space="preserve">requirements.txt, README e .gitignore</t>
   </si>
   <si>
-    <t xml:space="preserve">Docker (Dockerfile + docker-compose): roda com 1 comando e dados persistentes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docker compose up -d --build</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Script para iniciar o servidor (iniciar_servidor.bat)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Script de configuração das TVs atualizado para as URLs por slug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">setup_tv.bat</t>
+    <t xml:space="preserve">Docker (1 comando) + código em volume para atualizar sem rebuild</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scripts de iniciar servidor e configurar as TVs</t>
   </si>
   <si>
     <t xml:space="preserve">IDENTIDADE VISUAL</t>
@@ -152,103 +122,154 @@
     <t xml:space="preserve">Identidade</t>
   </si>
   <si>
-    <t xml:space="preserve">Logo do Grupo Flexível inserido (login, admin e TVs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paleta verde da marca aplicada nas três telas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Híbrida: verde + laranja p/ alertas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipografia Roboto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logo organizado em frontend/assets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tirado da raiz do projeto</t>
+    <t xml:space="preserve">Logo do Grupo Flexível nas telas (login, admin, TVs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paleta verde da marca + fonte Roboto</t>
   </si>
   <si>
     <t xml:space="preserve">Documento de identidade visual adaptado ao projeto</t>
   </si>
   <si>
-    <t xml:space="preserve">docs/IDENTIDADE_VISUAL.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TELA DAS TVs (DISPLAY)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remoção do cabeçalho do topo</t>
+    <t xml:space="preserve">GRADE DE PROGRAMAÇÃO (UNIFICADA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editor único 'Montar Grade' (substitui menus separados)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartões visuais: miniatura, arrastar p/ reordenar, editar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tempo de cada slide editável no próprio cartão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remoção do cabeçalho do topo no display</t>
   </si>
   <si>
     <t xml:space="preserve">Remoção completa do módulo de KPI</t>
   </si>
   <si>
-    <t xml:space="preserve">Não será utilizado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barra inferior configurável (construtor de barra)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cor da barra por código HEX ou RGB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Widget de data e hora com seleção de fuso horário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Widget de logo no rodapé (dimensionado à barra)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Widgets reordenáveis e com liga/desliga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monta a barra como quiser</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cotações de Dólar e Euro (USD/BRL e EUR/BRL) com atualização diária</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exige internet no servidor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PENDÊNCIAS – FASE 2 (do documento mestre)</t>
+    <t xml:space="preserve">CONTEÚDOS / MÍDIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mídia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagem, vídeo (MP4) e galeria de fotos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YouTube com player que avança no fim do vídeo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toca mudo (autoplay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDF exibido em tela cheia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tela cheia com fundo desfocado (sem cortar nem esticar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regras de upload: PNG, JPG, JPEG, MP4, PDF + dimensões recomendadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIBLIOTECA DE MÍDIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biblioteca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pastas: criar, navegar (caminho), enviar na pasta, excluir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mover arquivos arrastando (atualiza referências nos slides)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escolher da biblioteca ao montar a grade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BARRA INFERIOR (RODAPÉ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construtor de barra: cor (HEX/RGB) e ordem dos widgets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posicionar widgets: esquerda / centro / direita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altura da barra configurável</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logo no rodapé com upload e opção de fundo transparente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora com seleção de fuso horário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cotações Dólar e Euro (USD/BRL, EUR/BRL) diárias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ícones $ / €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Previsão do tempo por cidade (seleção exata por coordenadas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mín azul / máx vermelho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notícias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notícias por categoria: imagem + manchete + fonte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">via GNews</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 notícia por volta da grade + palavras proibidas (global)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDÊNCIAS – FASE 2</t>
   </si>
   <si>
     <t xml:space="preserve">Fase 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Grupos de telas (aplicar uma grade a um grupo inteiro)</t>
+    <t xml:space="preserve">Grupos de telas (aplicar grade a um grupo)</t>
   </si>
   <si>
     <t xml:space="preserve">Pendente</t>
   </si>
   <si>
-    <t xml:space="preserve">Próxima etapa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notícias por categoria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Captura de URL (print de páginas para exibir)</t>
+    <t xml:space="preserve">Captura de URL (print de páginas)</t>
   </si>
   <si>
     <t xml:space="preserve">Posts de redes sociais (Facebook)</t>
   </si>
   <si>
-    <t xml:space="preserve">Depende de credenciais externas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Banco de dados (hoje o conteúdo fica em arquivo JSON)</t>
+    <t xml:space="preserve">depende de API externa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banco de dados (hoje o conteúdo é arquivo JSON)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simular a grade antes de publicar</t>
   </si>
   <si>
     <t xml:space="preserve">Backup automático do conteúdo</t>
   </si>
   <si>
     <t xml:space="preserve">Troca de senha obrigatória no 1º acesso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testes automatizados formais</t>
   </si>
   <si>
     <t xml:space="preserve">CRONOGRAMA DE PROJETO – TV CORPORATIVA</t>
@@ -827,7 +848,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1294,15 +1315,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1327,8 +1348,8 @@
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="str">
-        <f aca="false">CONCATENATE("Concluídos: ",COUNTIF(D5:D47,"Concluído"),"   |   Pendentes: ",COUNTIF(D5:D47,"Pendente"),"   |   % concluído: ",TEXT(COUNTIF(D5:D47,"Concluído")/(COUNTIF(D5:D47,"Concluído")+COUNTIF(D5:D47,"Pendente")),"0%"))</f>
-        <v>Concluídos: 30   |   Pendentes: 7   |   % concluído: 81%</v>
+        <f aca="false">CONCATENATE("Concluídos: ",COUNTIF(D5:D59,"Concluído"),"   |   Pendentes: ",COUNTIF(D5:D59,"Pendente"),"   |   % concluído: ",TEXT(COUNTIF(D5:D59,"Concluído")/(COUNTIF(D5:D59,"Concluído")+COUNTIF(D5:D59,"Pendente")),"0%"))</f>
+        <v>Concluídos: 38   |   Pendentes: 8   |   % concluído: 83%</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1366,7 +1387,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
@@ -1382,11 +1403,9 @@
       <c r="E6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="n">
         <v>2</v>
       </c>
@@ -1394,7 +1413,7 @@
         <v>9</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>11</v>
@@ -1402,11 +1421,9 @@
       <c r="E7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F7" s="12"/>
+    </row>
+    <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
@@ -1414,7 +1431,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>11</v>
@@ -1422,11 +1439,9 @@
       <c r="E8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="n">
         <v>4</v>
       </c>
@@ -1434,7 +1449,7 @@
         <v>9</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>11</v>
@@ -1444,7 +1459,7 @@
       </c>
       <c r="F9" s="12"/>
     </row>
-    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
         <v>5</v>
       </c>
@@ -1452,7 +1467,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>11</v>
@@ -1462,45 +1477,45 @@
       </c>
       <c r="F10" s="8"/>
     </row>
-    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
+    <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="12" t="s">
+      <c r="B12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>11</v>
@@ -1508,19 +1523,17 @@
       <c r="E13" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F13" s="12"/>
+    </row>
+    <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
         <v>8</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>11</v>
@@ -1528,55 +1541,45 @@
       <c r="E14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F14" s="8"/>
+    </row>
+    <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="n">
         <v>9</v>
       </c>
       <c r="B15" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>28</v>
-      </c>
       <c r="D15" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F15" s="12"/>
     </row>
-    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="n">
+    <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="8"/>
-    </row>
-    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="n">
-        <v>11</v>
-      </c>
       <c r="B17" s="11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>11</v>
@@ -1586,15 +1589,15 @@
       </c>
       <c r="F17" s="12"/>
     </row>
-    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>11</v>
@@ -1604,25 +1607,33 @@
       </c>
       <c r="F18" s="8"/>
     </row>
-    <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19" s="12"/>
+    </row>
+    <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>11</v>
@@ -1632,33 +1643,25 @@
       </c>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="n">
+    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B22" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F21" s="12"/>
-    </row>
-    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>36</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>11</v>
@@ -1666,19 +1669,17 @@
       <c r="E22" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F22" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F22" s="8"/>
+    </row>
+    <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>11</v>
@@ -1688,15 +1689,15 @@
       </c>
       <c r="F23" s="12"/>
     </row>
-    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>11</v>
@@ -1704,13 +1705,11 @@
       <c r="E24" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F24" s="8" t="s">
-        <v>40</v>
-      </c>
+      <c r="F24" s="8"/>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1718,71 +1717,69 @@
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
     </row>
-    <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26" s="8"/>
+    </row>
+    <row r="27" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B26" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F26" s="8"/>
-    </row>
-    <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="n">
+      <c r="B27" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F27" s="12"/>
+    </row>
+    <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B27" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F27" s="12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="n">
+      <c r="B28" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F28" s="8"/>
+    </row>
+    <row r="29" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B28" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F28" s="8"/>
-    </row>
-    <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="n">
-        <v>21</v>
-      </c>
       <c r="B29" s="11" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>11</v>
@@ -1790,19 +1787,17 @@
       <c r="E29" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F29" s="12" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B30" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>11</v>
@@ -1810,13 +1805,11 @@
       <c r="E30" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F30" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -1824,15 +1817,15 @@
       <c r="E31" s="5"/>
       <c r="F31" s="5"/>
     </row>
-    <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>11</v>
@@ -1842,275 +1835,476 @@
       </c>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B33" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>12</v>
-      </c>
       <c r="F33" s="12" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="B34" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F34" s="8"/>
-    </row>
-    <row r="35" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="n">
+      <c r="B35" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F35" s="12"/>
+    </row>
+    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B35" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F35" s="12"/>
-    </row>
-    <row r="36" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="n">
+      <c r="B36" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F36" s="8"/>
+    </row>
+    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+    </row>
+    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="n">
         <v>27</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C36" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F36" s="8"/>
-    </row>
-    <row r="37" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="B37" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="D37" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F37" s="12"/>
-    </row>
-    <row r="38" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="n">
-        <v>29</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>52</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>24</v>
+      </c>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B39" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C39" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F39" s="12"/>
+    </row>
+    <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+    </row>
+    <row r="42" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F42" s="8"/>
+    </row>
+    <row r="43" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F43" s="12"/>
+    </row>
+    <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F44" s="8"/>
+    </row>
+    <row r="45" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F45" s="12"/>
+    </row>
+    <row r="46" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C46" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D39" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" s="10" t="s">
+      <c r="D46" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F39" s="12" t="s">
+      <c r="F46" s="8"/>
+    </row>
+    <row r="47" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47" s="12" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
+      <c r="D47" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F47" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-    </row>
-    <row r="41" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="B41" s="11" t="s">
+    </row>
+    <row r="48" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C41" s="12" t="s">
+      <c r="D48" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F48" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D41" s="13" t="s">
+    </row>
+    <row r="49" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="B49" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E41" s="10"/>
-      <c r="F41" s="12" t="s">
+      <c r="C49" s="12" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="n">
-        <v>32</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="C42" s="8" t="s">
+      <c r="D49" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F49" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="D42" s="13" t="s">
+    </row>
+    <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B50" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="E42" s="6"/>
-      <c r="F42" s="8"/>
-    </row>
-    <row r="43" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10" t="n">
-        <v>33</v>
-      </c>
-      <c r="B43" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C43" s="12" t="s">
+      <c r="C50" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="D43" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E43" s="10"/>
-      <c r="F43" s="12"/>
-    </row>
-    <row r="44" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="C44" s="8" t="s">
+      <c r="D50" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F50" s="8"/>
+    </row>
+    <row r="51" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="D44" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E44" s="6"/>
-      <c r="F44" s="8" t="s">
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+    </row>
+    <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B52" s="7" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="45" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="10" t="n">
-        <v>35</v>
-      </c>
-      <c r="B45" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C45" s="12" t="s">
+      <c r="C52" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D45" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E45" s="10"/>
-      <c r="F45" s="12"/>
-    </row>
-    <row r="46" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="C46" s="8" t="s">
+      <c r="D52" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="D46" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E46" s="6"/>
-      <c r="F46" s="8"/>
-    </row>
-    <row r="47" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="10" t="n">
-        <v>37</v>
-      </c>
-      <c r="B47" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C47" s="12" t="s">
+      <c r="E52" s="6"/>
+      <c r="F52" s="8"/>
+    </row>
+    <row r="53" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C53" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="D47" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E47" s="10"/>
-      <c r="F47" s="12"/>
+      <c r="D53" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E53" s="10"/>
+      <c r="F53" s="12"/>
+    </row>
+    <row r="54" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D54" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E54" s="6"/>
+      <c r="F54" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D55" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E55" s="10"/>
+      <c r="F55" s="12"/>
+    </row>
+    <row r="56" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D56" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E56" s="6"/>
+      <c r="F56" s="8"/>
+    </row>
+    <row r="57" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D57" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E57" s="10"/>
+      <c r="F57" s="12"/>
+    </row>
+    <row r="58" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D58" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E58" s="6"/>
+      <c r="F58" s="8"/>
+    </row>
+    <row r="59" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D59" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E59" s="10"/>
+      <c r="F59" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="12">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A25:F25"/>
     <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A51:F51"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2142,7 +2336,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -2155,7 +2349,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -2171,25 +2365,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="G3" s="17" t="s">
         <v>5</v>
       </c>
       <c r="H3" s="17" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="I3" s="17" t="s">
         <v>7</v>
@@ -2197,7 +2391,7 @@
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B4" s="18"/>
       <c r="C4" s="18"/>
@@ -2210,13 +2404,13 @@
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D5" s="21" t="n">
         <v>46196</v>
@@ -2235,18 +2429,18 @@
         <v>1</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="25" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D6" s="27" t="n">
         <v>46197</v>
@@ -2265,18 +2459,18 @@
         <v>1</v>
       </c>
       <c r="I6" s="26" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>46199</v>
@@ -2295,18 +2489,18 @@
         <v>1</v>
       </c>
       <c r="I7" s="20" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="25" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D8" s="27" t="n">
         <v>46201</v>
@@ -2325,18 +2519,18 @@
         <v>1</v>
       </c>
       <c r="I8" s="26" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D9" s="21" t="n">
         <v>46206</v>
@@ -2349,18 +2543,18 @@
         <v>2</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H9" s="24" t="n">
         <v>0.5</v>
       </c>
       <c r="I9" s="20" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B10" s="18"/>
       <c r="C10" s="18"/>
@@ -2373,13 +2567,13 @@
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D11" s="33" t="n">
         <v>46209</v>
@@ -2398,18 +2592,18 @@
         <v>1</v>
       </c>
       <c r="I11" s="32" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="36" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D12" s="38" t="n">
         <v>46212</v>
@@ -2428,18 +2622,18 @@
         <v>1</v>
       </c>
       <c r="I12" s="37" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="C13" s="32" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D13" s="33" t="n">
         <v>46216</v>
@@ -2458,18 +2652,18 @@
         <v>1</v>
       </c>
       <c r="I13" s="32" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="36" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D14" s="38" t="n">
         <v>46218</v>
@@ -2488,18 +2682,18 @@
         <v>1</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D15" s="33" t="n">
         <v>46224</v>
@@ -2518,18 +2712,18 @@
         <v>1</v>
       </c>
       <c r="I15" s="32" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="36" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C16" s="37" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D16" s="38" t="n">
         <v>46226</v>
@@ -2548,12 +2742,12 @@
         <v>1</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="B17" s="18"/>
       <c r="C17" s="18"/>
@@ -2566,13 +2760,13 @@
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="41" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B18" s="42" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D18" s="43" t="n">
         <v>46237</v>
@@ -2591,18 +2785,18 @@
         <v>1</v>
       </c>
       <c r="I18" s="42" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="46" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B19" s="47" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C19" s="47" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D19" s="48" t="n">
         <v>46241</v>
@@ -2621,18 +2815,18 @@
         <v>1</v>
       </c>
       <c r="I19" s="47" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="41" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B20" s="42" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C20" s="42" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D20" s="43" t="n">
         <v>46245</v>
@@ -2645,24 +2839,24 @@
         <v>9</v>
       </c>
       <c r="G20" s="30" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H20" s="45" t="n">
         <v>0.3</v>
       </c>
       <c r="I20" s="42" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="46" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="B21" s="47" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C21" s="47" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D21" s="48" t="n">
         <v>46253</v>
@@ -2675,24 +2869,24 @@
         <v>4</v>
       </c>
       <c r="G21" s="30" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H21" s="50" t="n">
         <v>0.3</v>
       </c>
       <c r="I21" s="47" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="41" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B22" s="42" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C22" s="42" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="D22" s="43" t="n">
         <v>46256</v>
@@ -2711,18 +2905,18 @@
         <v>1</v>
       </c>
       <c r="I22" s="42" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="46" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="B23" s="47" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C23" s="47" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D23" s="48" t="n">
         <v>46259</v>
@@ -2735,18 +2929,18 @@
         <v>2</v>
       </c>
       <c r="G23" s="30" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H23" s="50" t="n">
         <v>0.2</v>
       </c>
       <c r="I23" s="47" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="51" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B24" s="51"/>
       <c r="C24" s="52"/>
@@ -2762,19 +2956,19 @@
     </row>
     <row r="26" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="54" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B26" s="23" t="s">
         <v>11</v>
       </c>
       <c r="C26" s="30" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D26" s="55" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E26" s="56" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>